<commit_message>
Consolidated Con Law outline: add Week 11 Reading notes tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Con_Law_Outline_Consolidated.xlsx
+++ b/Con_Law_Outline_Consolidated.xlsx
@@ -31,11 +31,12 @@
     <sheet name="Week 9 - Class" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="Week 10 - Reading" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="Week 10 - Class" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Cases by Doctrine" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Midterm questions &amp; answers" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Week 11 - Reading" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Cases by Doctrine" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Midterm questions &amp; answers" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'Cases by Doctrine'!$A$1:$K$161</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'Cases by Doctrine'!$A$1:$K$161</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,7 +666,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -1003,6 +1004,9 @@
     <xf numFmtId="0" fontId="13" fillId="46" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="51" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10740,6 +10744,756 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="117" t="inlineStr">
+        <is>
+          <t>Case / Reading</t>
+        </is>
+      </c>
+      <c r="B1" s="117" t="inlineStr">
+        <is>
+          <t>Doctrine</t>
+        </is>
+      </c>
+      <c r="C1" s="117" t="inlineStr">
+        <is>
+          <t>Holding (what was decided)</t>
+        </is>
+      </c>
+      <c r="D1" s="117" t="inlineStr">
+        <is>
+          <t>Key principle / rule it shaped</t>
+        </is>
+      </c>
+      <c r="E1" s="117" t="inlineStr">
+        <is>
+          <t>Remember for the exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="112" t="inlineStr">
+        <is>
+          <t>The Federalist No. 39 (Madison, 1788)</t>
+        </is>
+      </c>
+      <c r="B2" s="111" t="inlineStr">
+        <is>
+          <t>Republican government; tenure of officers</t>
+        </is>
+      </c>
+      <c r="C2" s="111" t="inlineStr">
+        <is>
+          <t>N/A (reading)</t>
+        </is>
+      </c>
+      <c r="D2" s="111" t="inlineStr">
+        <is>
+          <t>A republic is a government that gets all its power directly or indirectly from the great body of the people, run by people who serve at pleasure, for a limited term, or during good behavior. It is ESSENTIAL that power come from the people as a whole, not a favored class; it is SUFFICIENT that officers are chosen directly or indirectly by the people. House = direct election; Senate, President and judges = indirect. Key line: 'The tenure of the ministerial offices generally, will be a subject of legal regulation.'</t>
+        </is>
+      </c>
+      <c r="E2" s="111" t="inlineStr">
+        <is>
+          <t>Slaughter dissent reads 'legal regulation' of tenure to mean Congress can limit removal. Majority: Madison meant only fixed TERMS for officers, still removable by the President in between.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="112" t="inlineStr">
+        <is>
+          <t>The Federalist No. 77 (Hamilton, 1788)</t>
+        </is>
+      </c>
+      <c r="B3" s="111" t="inlineStr">
+        <is>
+          <t>Appointments and removal</t>
+        </is>
+      </c>
+      <c r="C3" s="111" t="inlineStr">
+        <is>
+          <t>N/A (reading)</t>
+        </is>
+      </c>
+      <c r="D3" s="111" t="inlineStr">
+        <is>
+          <t>Senate consent 'would be necessary to displace as well as to appoint.' Selling point: a new President couldn't sweep out good officers, giving a 'steady administration'; the Senate is more stable than other branches.</t>
+        </is>
+      </c>
+      <c r="E3" s="111" t="inlineStr">
+        <is>
+          <t>Dissent's best founding quote against at-will removal. Majority: unclear whether 'displace' meant REMOVE or REPLACE; conflicts with Fed. 70 and 72; Hamilton said by 1793 (Pacificus No. 1) that removal is executive power.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="112" t="inlineStr">
+        <is>
+          <t>Letter, Rep. William Smith to Edward Rutledge (June 21, 1789)</t>
+        </is>
+      </c>
+      <c r="B4" s="111" t="inlineStr">
+        <is>
+          <t>Decision of 1789 — background</t>
+        </is>
+      </c>
+      <c r="C4" s="111" t="inlineStr">
+        <is>
+          <t>N/A (reading)</t>
+        </is>
+      </c>
+      <c r="D4" s="111" t="inlineStr">
+        <is>
+          <t>Describes the House's 4-day debate over giving the President the removal power ('the most important question'). Smith quoted Federalist No. 77 for his side; Rep. Benson then passed him a note saying 'Publius' (Hamilton) had changed his mind and now thought the President ALONE should remove at pleasure — while Hamilton was a candidate for Secretary of the Treasury.</t>
+        </is>
+      </c>
+      <c r="E4" s="111" t="inlineStr">
+        <is>
+          <t>Shows Hamilton's Fed. 77 view was disputed or abandoned even in 1789; cuts against relying on Fed. 77.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="112" t="inlineStr">
+        <is>
+          <t>Edmond v. United States (1997) (Scalia)</t>
+        </is>
+      </c>
+      <c r="B5" s="111" t="inlineStr">
+        <is>
+          <t>Appointments Clause — principal vs. inferior officers</t>
+        </is>
+      </c>
+      <c r="C5" s="111" t="inlineStr">
+        <is>
+          <t>Civilian judges of the Coast Guard Court of Criminal Appeals are INFERIOR officers, so the Secretary of Transportation (a head of department) could validly appoint them.</t>
+        </is>
+      </c>
+      <c r="D5" s="111" t="inlineStr">
+        <is>
+          <t>Appointments Clause: principal officers = President + Senate consent; Congress may vest appointment of inferior officers in the President alone, courts of law, or heads of departments ('Excepting Clause,' for administrative convenience). 'Significant authority' (Buckley) marks officer vs. employee, NOT principal vs. inferior. Test: an inferior officer has a SUPERIOR — work is 'directed and supervised at some level' by Senate-confirmed officers. Here: the Judge Advocate General sets rules and can remove the judges without cause; the Court of Appeals for the Armed Forces can reverse them. Key: they cannot render a FINAL decision for the U.S. unless other executive officers permit it.</t>
+        </is>
+      </c>
+      <c r="E5" s="111" t="inlineStr">
+        <is>
+          <t>Factors: who supervises, who can remove (removal = 'powerful tool for control'), whether decisions are final. Morrison's factors (limited duties, jurisdiction, tenure) aren't a definitive test. First Congress called department heads 'principal' and chief clerks 'inferior.' Purpose: accountability — blame for bad picks falls on President and Senate (Fed. 76, 77).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="112" t="inlineStr">
+        <is>
+          <t>Lucia v. SEC (2018) (Kagan, 7-2)</t>
+        </is>
+      </c>
+      <c r="B6" s="111" t="inlineStr">
+        <is>
+          <t>Appointments Clause — officer vs. employee</t>
+        </is>
+      </c>
+      <c r="C6" s="111" t="inlineStr">
+        <is>
+          <t>SEC administrative law judges are 'Officers of the United States.' Because SEC staff (not the Commission) hired them, they were unconstitutionally appointed.</t>
+        </is>
+      </c>
+      <c r="D6" s="111" t="inlineStr">
+        <is>
+          <t>Officer test: (1) a CONTINUING position established by law (Germaine — not 'occasional or temporary'); and (2) exercises SIGNIFICANT AUTHORITY under federal law (Buckley). Freytag (Tax Court special trial judges) controls: SEC ALJs take testimony, conduct trials, rule on evidence, and enforce discovery orders — same as STJs. A fortiori: if the SEC declines review, the ALJ's decision becomes final and is 'deemed the action of the Commission.' Remedy: a NEW hearing before a properly appointed official, and NOT the same ALJ (Elliot), even if later properly appointed.</t>
+        </is>
+      </c>
+      <c r="E6" s="111" t="inlineStr">
+        <is>
+          <t>Facts: Raymond Lucia, 'Buckets of Money' retirement strategy; ALJ Elliot imposed $300,000 penalty and lifetime bar. The Government switched sides; Court appointed amicus. Commission itself = 'head of department' and may appoint ALJs (inferior officers). Lack of contempt/jail power doesn't matter — ALJs can exclude parties and suspend attorneys.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="112" t="inlineStr">
+        <is>
+          <t>Lucia — Thomas concurrence (with Gorsuch); other opinions</t>
+        </is>
+      </c>
+      <c r="B7" s="111" t="inlineStr">
+        <is>
+          <t>Appointments Clause</t>
+        </is>
+      </c>
+      <c r="C7" s="111" t="inlineStr">
+        <is>
+          <t>Agreed the case is indistinguishable from Freytag.</t>
+        </is>
+      </c>
+      <c r="D7" s="111" t="inlineStr">
+        <is>
+          <t>Thomas: precedents say what is SUFFICIENT to be an officer but never what is NECESSARY; the Court can't decide every future case by comparison to Freytag. (Breyer concurred in part/dissented in part; Sotomayor with Ginsburg dissented.)</t>
+        </is>
+      </c>
+      <c r="E7" s="111" t="inlineStr">
+        <is>
+          <t>Know the vote (7-2 on officer status) and that the officer test remains open-ended.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="112" t="inlineStr">
+        <is>
+          <t>Myers (1926) and Humphrey's Executor (1935) — as recounted in Trump v. Slaughter</t>
+        </is>
+      </c>
+      <c r="B8" s="111" t="inlineStr">
+        <is>
+          <t>Removal power — background</t>
+        </is>
+      </c>
+      <c r="C8" s="111" t="inlineStr">
+        <is>
+          <t>Myers: President may fire a postmaster without the Senate's consent; the 1876 law requiring consent was unconstitutional. Humphrey's: FDR couldn't fire FTC Commissioner Humphrey without cause, because the FTC was then described as 'quasi-legislative' and 'quasi-judicial,' exercising 'no part of the executive power.'</t>
+        </is>
+      </c>
+      <c r="D8" s="111" t="inlineStr">
+        <is>
+          <t>Myers (Taft): executive power + Take Care Clause imply power to remove those 'for whom he can not continue to be responsible.' Humphrey's (Sutherland): the President is 'master in his own house' but can't impose control 'in the house of another.' Humphrey's was decided on 'Black Monday' (same day as Schechter and Radford). Morrison v. Olson (1988) later admitted the FTC exercised executive power 'to some degree' even in 1935.</t>
+        </is>
+      </c>
+      <c r="E8" s="111" t="inlineStr">
+        <is>
+          <t>Humphrey reportedly called the FTC a 'publicity bureau' spreading 'Socialistic propaganda'; FDR fired him with a one-line letter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="112" t="inlineStr">
+        <is>
+          <t>Trump v. Slaughter (2026) (Roberts, 6-3)</t>
+        </is>
+      </c>
+      <c r="B9" s="111" t="inlineStr">
+        <is>
+          <t>Presidential removal power</t>
+        </is>
+      </c>
+      <c r="C9" s="111" t="inlineStr">
+        <is>
+          <t>The FTC Act's for-cause removal protection for Commissioners ('inefficiency, neglect of duty, or malfeasance') violates the separation of powers. The President could fire Commissioner Slaughter at will. Reversed and remanded.</t>
+        </is>
+      </c>
+      <c r="D9" s="111" t="inlineStr">
+        <is>
+          <t>Rule: officers who exercise EXECUTIVE power in the President's name must be removable by him at will. Sources: Vesting Clause + Take Care Clause; unity of the executive (Fed. 70: plurality 'tends to conceal faults and destroy responsibility'); the 'Decision of 1789' (Madison: removal power keeps the 'chain of dependence'); practice of early Presidents (Washington through Jackson); Hennen, Parsons, Myers. Humphrey's: 'all that is left' is that an agency exercising NO executive power need not be removable at will — 'If anything more is left of Humphrey's, we overrule it.' Today's FTC is executive 'through and through': (1) legislative rules with force of law, (2) investigates and adjudicates in-house, (3) sues in federal court for injunctions and civil penalties (billions, e.g., $2.5B Amazon).</t>
+        </is>
+      </c>
+      <c r="E9" s="111" t="inlineStr">
+        <is>
+          <t>Facts: March 2025, Trump fired the two remaining Democratic Commissioners (Slaughter, Bedoya), citing Article II, not cause. District Court reinstated her under Humphrey's; D.C. Circuit refused a stay (Judge Rao dissented: no 'headless fourth branch'); Supreme Court stayed and granted cert before judgment. Rejects 'practice makes perfect': like Chadha's ~300 legislative vetoes, widespread practice doesn't make it constitutional. Stare decisis is weakest in constitutional cases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="112" t="inlineStr">
+        <is>
+          <t>Trump v. Slaughter — limits on the holding (Part III-B; Thomas did not join)</t>
+        </is>
+      </c>
+      <c r="B10" s="111" t="inlineStr">
+        <is>
+          <t>Removal power — open questions</t>
+        </is>
+      </c>
+      <c r="C10" s="111" t="inlineStr">
+        <is>
+          <t>Court decides only the FTC, which is in the 'heartland' of executive power.</t>
+        </is>
+      </c>
+      <c r="D10" s="111" t="inlineStr">
+        <is>
+          <t>Left open: (1) entities with no executive or sovereign power (e.g., Boy Scouts, Georgetown — congressionally chartered); (2) the Federal Reserve, to the extent it follows the tradition of the First and Second Banks of the U.S.; (3) tenure protections for judges of non-Article III courts (Tax Court, Court of Federal Claims). Footnote: Marbury's justice of the peace could have fixed tenure because he exercised JUDICIAL power, not executive.</t>
+        </is>
+      </c>
+      <c r="E10" s="111" t="inlineStr">
+        <is>
+          <t>Dissent: these carve-outs are ad hoc; also flags unresolved questions for inferior officers (Perkins) and the civil service, and mixed adjudicatory agencies like the NLRB and MSPB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="112" t="inlineStr">
+        <is>
+          <t>Trump v. Slaughter — Gorsuch concurrence</t>
+        </is>
+      </c>
+      <c r="B11" s="111" t="inlineStr">
+        <is>
+          <t>Removal power + nondelegation</t>
+        </is>
+      </c>
+      <c r="C11" s="111" t="inlineStr">
+        <is>
+          <t>Agrees with the majority.</t>
+        </is>
+      </c>
+      <c r="D11" s="111" t="inlineStr">
+        <is>
+          <t>Warns: independent agencies hold vast LEGISLATIVE and JUDICIAL power delegated by Congress, and now the President controls all of it. Asks whether Congress would have delegated so much had it known. The 'only sure path' is to restore legislative power to Congress and judicial power to the courts — i.e., revive nondelegation.</t>
+        </is>
+      </c>
+      <c r="E11" s="111" t="inlineStr">
+        <is>
+          <t>Links removal (Slaughter) to nondelegation (Gundy dissent) and major questions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="112" t="inlineStr">
+        <is>
+          <t>Trump v. Slaughter — Sotomayor dissent (with Kagan, Jackson)</t>
+        </is>
+      </c>
+      <c r="B12" s="111" t="inlineStr">
+        <is>
+          <t>Removal power</t>
+        </is>
+      </c>
+      <c r="C12" s="111" t="inlineStr">
+        <is>
+          <t>Would uphold the FTC's for-cause protection under Humphrey's.</t>
+        </is>
+      </c>
+      <c r="D12" s="111" t="inlineStr">
+        <is>
+          <t>(1) Stare decisis: 90 years of precedent; 'profoundly easy case.' (2) 140 years of practice (ICC 1887, Board of General Appraisers 1890, Fed 1913, FTC 1914), approved by Presidents (Lincoln signed the Comptroller of the Currency law). (3) Text: the Constitution is silent on removal; Congress creates offices; Take Care 'speaks of duty, not power.' (4) Decision of 1789 decided only that the SENATE has no role in removal, not that Congress can't set causes (Bowsher distinction). (5) Fed. 77 and 39; Story, Kent, Webster, Clay, Calhoun. (6) Values besides accountability: stability, impartiality, expertise.</t>
+        </is>
+      </c>
+      <c r="E12" s="111" t="inlineStr">
+        <is>
+          <t>Majority's reply: Chadha shows long practice can't save an unconstitutional structure; the dissent would discard Myers itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="112" t="inlineStr">
+        <is>
+          <t>CRS, Congress's Authority to Influence and Control Executive Branch Agencies (2023)</t>
+        </is>
+      </c>
+      <c r="B13" s="111" t="inlineStr">
+        <is>
+          <t>Nondelegation — overview</t>
+        </is>
+      </c>
+      <c r="C13" s="111" t="inlineStr">
+        <is>
+          <t>N/A (reading)</t>
+        </is>
+      </c>
+      <c r="D13" s="111" t="inlineStr">
+        <is>
+          <t>Agencies have only the power Congress delegates; Congress can expand, narrow, sunset, or override it by statute. Nondelegation doctrine (separation of powers) bars Congress from giving away its core legislative function, but the test is lenient: Congress need only supply an 'INTELLIGIBLE PRINCIPLE' (J.W. Hampton, 1928). No law struck down on this ground since 1935 (Schechter, Panama Refining). 'Public interest' (NBC) and 'fair and equitable' (Yakus) standards have passed. Congress's tools: triggering conditions/factual findings, report-and-wait provisions, joint resolutions of disapproval (expedited procedures), and proposals that take effect only if enacted.</t>
+        </is>
+      </c>
+      <c r="E13" s="111" t="inlineStr">
+        <is>
+          <t>Contrast: appointment/removal doctrines stop Congress from encroaching on the executive; nondelegation stops Congress from giving its power away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="112" t="inlineStr">
+        <is>
+          <t>A.L.A. Schechter Poultry Corp. v. United States (1935) (Hughes, unanimous)</t>
+        </is>
+      </c>
+      <c r="B14" s="111" t="inlineStr">
+        <is>
+          <t>Nondelegation</t>
+        </is>
+      </c>
+      <c r="C14" s="111" t="inlineStr">
+        <is>
+          <t>NIRA §3 (letting the President approve or write 'codes of fair competition') was an unconstitutional delegation of legislative power; convictions under the Live Poultry Code reversed. (Also: Congress couldn't regulate these intrastate sales — 'indirect' effects on commerce.)</t>
+        </is>
+      </c>
+      <c r="D14" s="111" t="inlineStr">
+        <is>
+          <t>Congress may leave subordinate rules and fact-finding to others within prescribed limits, but may not transfer its essential legislative function. 'Fair competition' was undefined and far broader than common-law 'unfair competition' or the FTC Act's 'unfair methods of competition' (which had a quasi-judicial process, findings and judicial review). The only standards were the Act's broad policy goals, so the President's discretion was 'virtually unfettered.' Congress can't let trade groups write laws either.</t>
+        </is>
+      </c>
+      <c r="E14" s="111" t="inlineStr">
+        <is>
+          <t>Facts: Brooklyn kosher poultry slaughterhouses; 'straight killing' rule barred customers from picking individual chickens; convicted on counts including selling an 'unfit' chicken and wage/hour violations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="112" t="inlineStr">
+        <is>
+          <t>Schechter — Cardozo concurrence (with Stone)</t>
+        </is>
+      </c>
+      <c r="B15" s="111" t="inlineStr">
+        <is>
+          <t>Nondelegation</t>
+        </is>
+      </c>
+      <c r="C15" s="111" t="inlineStr">
+        <is>
+          <t>Concurs.</t>
+        </is>
+      </c>
+      <c r="D15" s="111" t="inlineStr">
+        <is>
+          <t>The power is 'not canalized within banks that keep it from overflowing'; it is a 'roving commission to inquire into evils and upon discovery correct them.' If 'fair' means anything good for business, 'This is delegation running riot.' Delegation to find and stop UNFAIR practices (like the FTC) would be fine. Also invalid under the Commerce Clause: 'Activities local in their immediacy do not become interstate and national because of distant repercussions.'</t>
+        </is>
+      </c>
+      <c r="E15" s="111" t="inlineStr">
+        <is>
+          <t>Most-quoted lines: 'delegation running riot'; 'roving commission'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="112" t="inlineStr">
+        <is>
+          <t>Gundy v. United States (2019) (Kagan plurality, 5-3)</t>
+        </is>
+      </c>
+      <c r="B16" s="111" t="inlineStr">
+        <is>
+          <t>Nondelegation — intelligible principle</t>
+        </is>
+      </c>
+      <c r="C16" s="111" t="inlineStr">
+        <is>
+          <t>SORNA §20913(d), letting the Attorney General 'specify the applicability' of registration requirements to pre-Act sex offenders, is a constitutional delegation.</t>
+        </is>
+      </c>
+      <c r="D16" s="111" t="inlineStr">
+        <is>
+          <t>Nondelegation analysis begins (and often almost ends) with statutory interpretation. Read in context (the 'comprehensive' national system in the purpose clause; definition of 'sex offender' as one who 'WAS convicted'; Reynolds), the statute requires the AG to apply SORNA to pre-Act offenders AS SOON AS FEASIBLE — discretion only over transitional feasibility issues. That is 'distinctly small-bore.' Only twice (both in 1935) has the Court struck a delegation. 'If SORNA's delegation is unconstitutional, then most of Government is unconstitutional.'</t>
+        </is>
+      </c>
+      <c r="E16" s="111" t="inlineStr">
+        <is>
+          <t>Facts: Herman Gundy, convicted in Maryland before SORNA (2006), failed to register in New York; faced up to 10 years. Kavanaugh did not participate; Alito's vote made 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="112" t="inlineStr">
+        <is>
+          <t>Gundy — Alito concurrence in the judgment</t>
+        </is>
+      </c>
+      <c r="B17" s="111" t="inlineStr">
+        <is>
+          <t>Nondelegation</t>
+        </is>
+      </c>
+      <c r="C17" s="111" t="inlineStr">
+        <is>
+          <t>Votes to affirm.</t>
+        </is>
+      </c>
+      <c r="D17" s="111" t="inlineStr">
+        <is>
+          <t>Would support reconsidering the intelligible-principle approach if a majority were willing; but it would be 'freakish' to single out this statute while the current test stands.</t>
+        </is>
+      </c>
+      <c r="E17" s="111" t="inlineStr">
+        <is>
+          <t>Signals five Justices (Alito + the 3 dissenters + later Kavanaugh) may revisit nondelegation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="112" t="inlineStr">
+        <is>
+          <t>Gundy — Gorsuch dissent (with Roberts, Thomas)</t>
+        </is>
+      </c>
+      <c r="B18" s="111" t="inlineStr">
+        <is>
+          <t>Nondelegation</t>
+        </is>
+      </c>
+      <c r="C18" s="111" t="inlineStr">
+        <is>
+          <t>Would hold the delegation unconstitutional.</t>
+        </is>
+      </c>
+      <c r="D18" s="111" t="inlineStr">
+        <is>
+          <t>The statute lets the nation's chief prosecutor write his own criminal code for ~500,000 people. Founders' reasons for hard lawmaking: liberty, deliberation, protecting minorities, fair notice, accountability (Locke: legislature 'cannot transfer the power of making laws'). Proposed test — Congress may: (1) make the policy and let others 'fill up the details' (Wayman v. Southard); (2) make a rule's application depend on executive FACT-FINDING (Cargo of the Brig Aurora); (3) assign non-legislative powers the executive already has (e.g., foreign affairs). The 'intelligible principle' phrase was a 'mutated' misreading of J.W. Hampton. Major questions doctrine is nondelegation under another name. Different AGs applied SORNA differently — proof of policymaking.</t>
+        </is>
+      </c>
+      <c r="E18" s="111" t="inlineStr">
+        <is>
+          <t>Pair with Gorsuch's Slaughter concurrence; 'Hopes and dreams are not laws.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="112" t="inlineStr">
+        <is>
+          <t>FCC v. Consumers' Research — Kavanaugh concurrence (question in reader)</t>
+        </is>
+      </c>
+      <c r="B19" s="111" t="inlineStr">
+        <is>
+          <t>Nondelegation</t>
+        </is>
+      </c>
+      <c r="C19" s="111" t="inlineStr">
+        <is>
+          <t>N/A (question)</t>
+        </is>
+      </c>
+      <c r="D19" s="111" t="inlineStr">
+        <is>
+          <t>Kavanaugh: 'the intelligible principle test is not toothless,' yet it 'has historically not packed much punch'; the President 'must act within the confines set by Congress.'</t>
+        </is>
+      </c>
+      <c r="E19" s="111" t="inlineStr">
+        <is>
+          <t>Reader asks: how much 'tooth' is that? Likely answer: little on its own — the real limits come from statutory interpretation and major questions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="112" t="inlineStr">
+        <is>
+          <t>Alabama Ass'n of Realtors v. HHS (2021) (per curiam)</t>
+        </is>
+      </c>
+      <c r="B20" s="111" t="inlineStr">
+        <is>
+          <t>Major questions doctrine</t>
+        </is>
+      </c>
+      <c r="C20" s="111" t="inlineStr">
+        <is>
+          <t>Vacated the stay; the CDC's nationwide COVID-19 eviction moratorium exceeded its authority under §361(a) of the Public Health Service Act.</t>
+        </is>
+      </c>
+      <c r="D20" s="111" t="inlineStr">
+        <is>
+          <t>Read the two sentences together: the second lists measures (inspection, fumigation, disinfection, pest extermination, destroying infected animals) that directly target disease; evictions affect spread only indirectly. Even if ambiguous, Congress must speak clearly for powers of 'vast economic and political significance': 80% of the country, 6-17 million tenants, ~$50B in rental aid, intrudes on state landlord-tenant law and the right to exclude. 'A wafer-thin reed.' 'Our system does not permit agencies to act unlawfully even in pursuit of desirable ends' (citing Youngstown). If the moratorium is to continue, Congress must authorize it.</t>
+        </is>
+      </c>
+      <c r="E20" s="111" t="inlineStr">
+        <is>
+          <t>Congress's own moratorium lapsed in July 2020; CDC kept extending it; criminal penalties up to $250,000 and 1 year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="112" t="inlineStr">
+        <is>
+          <t>Alabama Realtors — Breyer dissent (with Sotomayor, Kagan)</t>
+        </is>
+      </c>
+      <c r="B21" s="111" t="inlineStr">
+        <is>
+          <t>Major questions doctrine</t>
+        </is>
+      </c>
+      <c r="C21" s="111" t="inlineStr">
+        <is>
+          <t>Would leave the stay in place.</t>
+        </is>
+      </c>
+      <c r="D21" s="111" t="inlineStr">
+        <is>
+          <t>The first sentence broadly authorizes measures 'necessary' to stop disease; the second ('and other measures') expands, not limits. The order was tailored to high-transmission counties with tenant attestations. Equities and the Delta variant favor the CDC; emergency docket is the wrong place to decide.</t>
+        </is>
+      </c>
+      <c r="E21" s="111" t="inlineStr">
+        <is>
+          <t>Know the stay factors (Nken): likelihood of success, irreparable harm, harm to others, public interest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="112" t="inlineStr">
+        <is>
+          <t>West Virginia v. EPA (2022) + CRS, The Major Questions Doctrine (2022)</t>
+        </is>
+      </c>
+      <c r="B22" s="111" t="inlineStr">
+        <is>
+          <t>Major questions doctrine</t>
+        </is>
+      </c>
+      <c r="C22" s="111" t="inlineStr">
+        <is>
+          <t>West Virginia: EPA lacked clear authority (a 'previously little-used backwater' provision) to restructure the nation's energy mix.</t>
+        </is>
+      </c>
+      <c r="D22" s="111" t="inlineStr">
+        <is>
+          <t>First express use of 'major questions doctrine' in a majority opinion. Two steps: (1) the claimed authority involves vast economic and political significance; (2) Congress hasn't CLEARLY authorized it. A 'merely plausible textual basis' isn't enough; Congress doesn't hide elephants in mouseholes ('modest, vague, subtle, or ambiguous' language). Contrast Massachusetts v. EPA (2007), which rejected EPA's major-questions argument and held it could regulate vehicle greenhouse gases.</t>
+        </is>
+      </c>
+      <c r="E22" s="111" t="inlineStr">
+        <is>
+          <t>Reader question: the doctrine lets the Court AVOID the constitutional nondelegation question by reading the statute narrowly (Gorsuch: nondelegation 'by different names').</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="112" t="inlineStr">
+        <is>
+          <t>CRS, Executive Privilege and Presidential Communications: Judicial Principles (2022)</t>
+        </is>
+      </c>
+      <c r="B23" s="111" t="inlineStr">
+        <is>
+          <t>Executive privilege — overview</t>
+        </is>
+      </c>
+      <c r="C23" s="111" t="inlineStr">
+        <is>
+          <t>N/A (reading)</t>
+        </is>
+      </c>
+      <c r="D23" s="111" t="inlineStr">
+        <is>
+          <t>Not one privilege but several: state secrets; presidential communications (President and close advisers, for presidential decisionmaking); deliberative process (within agencies); law enforcement. The privilege is QUALIFIED, not absolute, and implied from Article II and separation of powers. Disputes with Congress are mostly resolved by negotiation and accommodation; the Supreme Court has never decided executive privilege against a congressional subpoena; courts prefer to avoid such disputes.</t>
+        </is>
+      </c>
+      <c r="E23" s="111" t="inlineStr">
+        <is>
+          <t>Executive branch reads the privilege broadly; Congress narrowly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="112" t="inlineStr">
+        <is>
+          <t>Watergate background and the 'smoking gun' tape (June 23, 1972)</t>
+        </is>
+      </c>
+      <c r="B24" s="111" t="inlineStr">
+        <is>
+          <t>Executive privilege — facts</t>
+        </is>
+      </c>
+      <c r="C24" s="111" t="inlineStr">
+        <is>
+          <t>N/A (reading)</t>
+        </is>
+      </c>
+      <c r="D24" s="111" t="inlineStr">
+        <is>
+          <t>Watergate break-in (June 17, 1972). Senate Watergate Committee and Special Prosecutor Archibald Cox both subpoenaed White House tapes after Alexander Butterfield revealed the Oval Office taping system; Nixon refused both (July 25, 1973). On the 'smoking gun' tape, Haldeman proposes having the CIA (Walters) tell FBI Director Pat Gray to 'stay the hell out of this,' and Nixon agrees — obstruction of the FBI investigation.</t>
+        </is>
+      </c>
+      <c r="E24" s="111" t="inlineStr">
+        <is>
+          <t>Release of this tape after U.S. v. Nixon led directly to resignation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="112" t="inlineStr">
+        <is>
+          <t>United States v. Nixon (1974) (Burger, 8-0; Rehnquist recused)</t>
+        </is>
+      </c>
+      <c r="B25" s="111" t="inlineStr">
+        <is>
+          <t>Executive privilege</t>
+        </is>
+      </c>
+      <c r="C25" s="111" t="inlineStr">
+        <is>
+          <t>The President must comply with a subpoena for tapes needed in a criminal trial; his generalized claim of privilege yields. Affirmed the order for in camera review by the District Court.</t>
+        </is>
+      </c>
+      <c r="D25" s="111" t="inlineStr">
+        <is>
+          <t>(1) Justiciable: Marbury — 'it is emphatically the province and duty of the judicial department to say what the law is,' including the scope of executive privilege. (2) A PRESUMPTIVE privilege for presidential communications exists, rooted in Article II and separation of powers (candor in advice), though not in the text (McCulloch: implied powers). (3) Not ABSOLUTE: a generalized interest in confidentiality must yield to the 'demonstrated, specific need for evidence in a pending criminal trial' (due process, Sixth Amendment compulsory process; 'the public has a right to every man's evidence'). (4) Greater deference for military, diplomatic or national-security secrets. (5) Court must review in camera and protect irrelevant material (Burr: don't treat the President as 'an ordinary individual').</t>
+        </is>
+      </c>
+      <c r="E25" s="111" t="inlineStr">
+        <is>
+          <t>Facts: Nixon named an unindicted coconspirator; Special Prosecutor (Jaworski) subpoenaed tapes for the Mitchell trial. Footnote 19: Court did NOT decide civil cases, congressional demands, or state secrets. Nixon resigned Aug. 8-9, 1974.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="112" t="inlineStr">
+        <is>
+          <t>Nixon's resignation address (Aug. 8, 1974)</t>
+        </is>
+      </c>
+      <c r="B26" s="111" t="inlineStr">
+        <is>
+          <t>Executive privilege — aftermath</t>
+        </is>
+      </c>
+      <c r="C26" s="111" t="inlineStr">
+        <is>
+          <t>N/A (reading)</t>
+        </is>
+      </c>
+      <c r="D26" s="111" t="inlineStr">
+        <is>
+          <t>Nixon resigned effective noon Aug. 9, 1974, saying he lacked the congressional support needed to govern; Vice President Ford was sworn in.</t>
+        </is>
+      </c>
+      <c r="E26" s="111" t="inlineStr">
+        <is>
+          <t>Context only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="112" t="inlineStr">
+        <is>
+          <t>Dellums v. Powell (D.C. Cir. 1977)</t>
+        </is>
+      </c>
+      <c r="B27" s="111" t="inlineStr">
+        <is>
+          <t>Executive privilege — civil cases</t>
+        </is>
+      </c>
+      <c r="C27" s="111" t="inlineStr">
+        <is>
+          <t>A former President's privilege claim in a civil damages suit is subject to a BALANCING test; here it was overcome, with a protective order against public disclosure.</t>
+        </is>
+      </c>
+      <c r="D27" s="111" t="inlineStr">
+        <is>
+          <t>A civil litigant must show a 'substantial' and 'specific' need beyond the routine desire for relevant discovery; usually that won't be met. A FORMER President's claim gets less weight than an incumbent's.</t>
+        </is>
+      </c>
+      <c r="E27" s="111" t="inlineStr">
+        <is>
+          <t>Facts: 1971 'May Day' antiwar arrests; plaintiffs sought Oval Office tapes. Extends U.S. v. Nixon's balancing from criminal to civil cases.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -19645,7 +20399,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Cases by Doctrine: store week numbers as numbers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Con_Law_Outline_Consolidated.xlsx
+++ b/Con_Law_Outline_Consolidated.xlsx
@@ -12183,10 +12183,8 @@
           <t>Appointments &amp; removal</t>
         </is>
       </c>
-      <c r="C13" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C13" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D13" s="99" t="inlineStr">
         <is>
@@ -12241,10 +12239,8 @@
           <t>Appointments &amp; removal</t>
         </is>
       </c>
-      <c r="C14" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C14" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D14" s="99" t="inlineStr">
         <is>
@@ -12686,10 +12682,8 @@
           <t>Executive power</t>
         </is>
       </c>
-      <c r="C22" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C22" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D22" s="99" t="inlineStr">
         <is>
@@ -12745,10 +12739,8 @@
           <t>Executive power</t>
         </is>
       </c>
-      <c r="C23" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C23" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D23" s="99" t="inlineStr">
         <is>
@@ -12804,10 +12796,8 @@
           <t>Executive power</t>
         </is>
       </c>
-      <c r="C24" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C24" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D24" s="99" t="inlineStr">
         <is>
@@ -12859,10 +12849,8 @@
         </is>
       </c>
       <c r="B25" s="99" t="n"/>
-      <c r="C25" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C25" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D25" s="99" t="inlineStr">
         <is>
@@ -12913,10 +12901,8 @@
         </is>
       </c>
       <c r="B26" s="99" t="n"/>
-      <c r="C26" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C26" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D26" s="99" t="inlineStr">
         <is>
@@ -12968,10 +12954,8 @@
         </is>
       </c>
       <c r="B27" s="99" t="n"/>
-      <c r="C27" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C27" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D27" s="99" t="inlineStr">
         <is>
@@ -13022,10 +13006,8 @@
         </is>
       </c>
       <c r="B28" s="99" t="n"/>
-      <c r="C28" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C28" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D28" s="99" t="inlineStr">
         <is>
@@ -13081,10 +13063,8 @@
           <t>Appointments &amp; removal</t>
         </is>
       </c>
-      <c r="C29" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C29" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D29" s="99" t="inlineStr">
         <is>
@@ -13141,10 +13121,8 @@
           <t>Major questions &amp; nondelegation</t>
         </is>
       </c>
-      <c r="C30" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C30" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D30" s="99" t="inlineStr">
         <is>
@@ -13796,10 +13774,8 @@
           <t>Executive privilege</t>
         </is>
       </c>
-      <c r="C42" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C42" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D42" s="99" t="inlineStr">
         <is>
@@ -17887,10 +17863,8 @@
           <t>Major questions &amp; nondelegation</t>
         </is>
       </c>
-      <c r="C117" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C117" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D117" s="99" t="inlineStr">
         <is>
@@ -20764,10 +20738,8 @@
           <t>Executive power; Treaties &amp; executive agreements</t>
         </is>
       </c>
-      <c r="C168" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C168" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D168" s="99" t="inlineStr">
         <is>
@@ -20823,10 +20795,8 @@
           <t>Appointments &amp; removal</t>
         </is>
       </c>
-      <c r="C169" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C169" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D169" s="99" t="inlineStr">
         <is>
@@ -20881,10 +20851,8 @@
           <t>Separation of powers</t>
         </is>
       </c>
-      <c r="C170" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C170" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D170" s="99" t="inlineStr">
         <is>
@@ -20940,10 +20908,8 @@
           <t>Commerce Clause</t>
         </is>
       </c>
-      <c r="C171" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C171" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D171" s="99" t="inlineStr">
         <is>
@@ -20995,10 +20961,8 @@
         </is>
       </c>
       <c r="B172" s="99" t="n"/>
-      <c r="C172" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C172" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D172" s="99" t="inlineStr">
         <is>
@@ -21049,10 +21013,8 @@
         </is>
       </c>
       <c r="B173" s="99" t="n"/>
-      <c r="C173" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C173" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D173" s="99" t="inlineStr">
         <is>
@@ -21104,10 +21066,8 @@
         </is>
       </c>
       <c r="B174" s="99" t="n"/>
-      <c r="C174" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C174" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D174" s="99" t="inlineStr">
         <is>
@@ -21157,10 +21117,8 @@
         </is>
       </c>
       <c r="B175" s="99" t="n"/>
-      <c r="C175" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C175" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D175" s="99" t="inlineStr">
         <is>
@@ -21212,10 +21170,8 @@
         </is>
       </c>
       <c r="B176" s="99" t="n"/>
-      <c r="C176" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C176" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D176" s="99" t="inlineStr">
         <is>
@@ -21265,10 +21221,8 @@
         </is>
       </c>
       <c r="B177" s="99" t="n"/>
-      <c r="C177" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C177" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D177" s="99" t="inlineStr">
         <is>
@@ -21320,10 +21274,8 @@
         </is>
       </c>
       <c r="B178" s="99" t="n"/>
-      <c r="C178" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C178" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D178" s="99" t="inlineStr">
         <is>
@@ -21768,10 +21720,8 @@
           <t>Executive power; Major questions &amp; nondelegation</t>
         </is>
       </c>
-      <c r="C186" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C186" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D186" s="99" t="inlineStr">
         <is>
@@ -21827,10 +21777,8 @@
           <t>Executive power</t>
         </is>
       </c>
-      <c r="C187" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C187" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D187" s="99" t="inlineStr">
         <is>
@@ -21885,10 +21833,8 @@
           <t>Executive power</t>
         </is>
       </c>
-      <c r="C188" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C188" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D188" s="99" t="inlineStr">
         <is>
@@ -21944,10 +21890,8 @@
           <t>Executive power</t>
         </is>
       </c>
-      <c r="C189" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C189" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D189" s="99" t="inlineStr">
         <is>
@@ -22003,10 +21947,8 @@
           <t>Executive power</t>
         </is>
       </c>
-      <c r="C190" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C190" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D190" s="99" t="inlineStr">
         <is>
@@ -22062,10 +22004,8 @@
           <t>Separation of powers</t>
         </is>
       </c>
-      <c r="C191" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C191" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D191" s="99" t="inlineStr">
         <is>
@@ -22121,10 +22061,8 @@
           <t>Treaties &amp; executive agreements; Major questions &amp; nondelegation</t>
         </is>
       </c>
-      <c r="C192" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C192" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D192" s="99" t="inlineStr">
         <is>
@@ -22176,10 +22114,8 @@
         </is>
       </c>
       <c r="B193" s="99" t="n"/>
-      <c r="C193" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C193" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D193" s="99" t="inlineStr">
         <is>
@@ -22234,10 +22170,8 @@
           <t>Separation of powers</t>
         </is>
       </c>
-      <c r="C194" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C194" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D194" s="99" t="inlineStr">
         <is>
@@ -22293,10 +22227,8 @@
           <t>Separation of powers</t>
         </is>
       </c>
-      <c r="C195" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C195" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D195" s="99" t="inlineStr">
         <is>
@@ -22348,10 +22280,8 @@
         </is>
       </c>
       <c r="B196" s="99" t="n"/>
-      <c r="C196" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C196" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D196" s="99" t="inlineStr">
         <is>
@@ -22406,10 +22336,8 @@
           <t>Treaties &amp; executive agreements</t>
         </is>
       </c>
-      <c r="C197" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C197" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D197" s="99" t="inlineStr">
         <is>
@@ -22464,10 +22392,8 @@
           <t>Treaties &amp; executive agreements</t>
         </is>
       </c>
-      <c r="C198" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C198" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D198" s="99" t="inlineStr">
         <is>
@@ -22523,10 +22449,8 @@
           <t>Treaties &amp; executive agreements</t>
         </is>
       </c>
-      <c r="C199" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C199" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D199" s="99" t="inlineStr">
         <is>
@@ -22582,10 +22506,8 @@
           <t>Treaties &amp; executive agreements</t>
         </is>
       </c>
-      <c r="C200" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C200" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D200" s="99" t="inlineStr">
         <is>
@@ -22641,10 +22563,8 @@
           <t>Foundations &amp; interpretation</t>
         </is>
       </c>
-      <c r="C201" s="99" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C201" s="99" t="n">
+        <v>10</v>
       </c>
       <c r="D201" s="99" t="inlineStr">
         <is>
@@ -22699,10 +22619,8 @@
           <t>Foundations &amp; interpretation</t>
         </is>
       </c>
-      <c r="C202" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C202" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D202" s="99" t="inlineStr">
         <is>
@@ -22754,10 +22672,8 @@
         </is>
       </c>
       <c r="B203" s="99" t="n"/>
-      <c r="C203" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C203" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D203" s="99" t="inlineStr">
         <is>
@@ -22808,10 +22724,8 @@
         </is>
       </c>
       <c r="B204" s="99" t="n"/>
-      <c r="C204" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C204" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D204" s="99" t="inlineStr">
         <is>
@@ -22862,10 +22776,8 @@
         </is>
       </c>
       <c r="B205" s="99" t="n"/>
-      <c r="C205" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C205" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D205" s="99" t="inlineStr">
         <is>
@@ -22918,10 +22830,8 @@
         </is>
       </c>
       <c r="B206" s="99" t="n"/>
-      <c r="C206" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C206" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D206" s="99" t="inlineStr">
         <is>
@@ -22974,10 +22884,8 @@
         </is>
       </c>
       <c r="B207" s="99" t="n"/>
-      <c r="C207" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C207" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D207" s="99" t="inlineStr">
         <is>
@@ -23033,10 +22941,8 @@
           <t>Separation of powers</t>
         </is>
       </c>
-      <c r="C208" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C208" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D208" s="99" t="inlineStr">
         <is>
@@ -23093,10 +22999,8 @@
           <t>Major questions &amp; nondelegation</t>
         </is>
       </c>
-      <c r="C209" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C209" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D209" s="99" t="inlineStr">
         <is>
@@ -23147,10 +23051,8 @@
         </is>
       </c>
       <c r="B210" s="99" t="n"/>
-      <c r="C210" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C210" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D210" s="99" t="inlineStr">
         <is>
@@ -23202,10 +23104,8 @@
         </is>
       </c>
       <c r="B211" s="99" t="n"/>
-      <c r="C211" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C211" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D211" s="99" t="inlineStr">
         <is>
@@ -23257,10 +23157,8 @@
         </is>
       </c>
       <c r="B212" s="99" t="n"/>
-      <c r="C212" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C212" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D212" s="99" t="inlineStr">
         <is>
@@ -23314,10 +23212,8 @@
           <t>Judicial review &amp; federal jurisdiction</t>
         </is>
       </c>
-      <c r="C213" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C213" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D213" s="99" t="inlineStr">
         <is>
@@ -23370,10 +23266,8 @@
         </is>
       </c>
       <c r="B214" s="99" t="n"/>
-      <c r="C214" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C214" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D214" s="99" t="inlineStr">
         <is>
@@ -23423,10 +23317,8 @@
         </is>
       </c>
       <c r="B215" s="99" t="n"/>
-      <c r="C215" s="99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C215" s="99" t="n">
+        <v>11</v>
       </c>
       <c r="D215" s="99" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Con Law outline: add Week 8 class notes (10/15)
Replaces the empty Week 8 - Class placeholder with 19 topics: Commerce
Clause after 1937 (Lopez, Morrison, Raich), NFIB (activity/inactivity,
tax, Medicaid coercion), Phomma, Protho, Chavarria, Bonner, Brutus vs.
Federalist 44, the Tenth Amendment, the 1791 bank debate, McCulloch,
and the dormant Commerce Clause (Brown-Forman, Dean Milk, Pike, Reeves).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Con_Law_Outline_Consolidated.xlsx
+++ b/Con_Law_Outline_Consolidated.xlsx
@@ -9508,7 +9508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -9530,13 +9530,283 @@
     <row r="2">
       <c r="A2" s="112" t="inlineStr">
         <is>
-          <t>No class notes on file yet</t>
+          <t>Commerce Clause after 1937: Lopez, Morrison, Raich</t>
         </is>
       </c>
       <c r="B2" s="111" t="inlineStr">
         <is>
-          <t>• Your outline has no class notes labeled Week 8.
-• Send them and they will be added here.</t>
+          <t>• After 1937 there seemed to be no real limit on the commerce power, other than other parts of the Constitution (like the First Amendment).
+• Lopez (1995): Congress went too far for the first time; people disagreed about whether it was a return to pre-1937 limits, a modest change, or meaningless.
+• Morrison followed and supported the idea of a sea change.
+• Gonzales v. Raich upheld regulating home-grown marijuana, like Wickard (never overruled): in the aggregate it substantially affects interstate commerce.
+• Difference: the Lopez law wasn't part of a larger economic regulation; Raich's was part of a comprehensive scheme.
+• After Raich, Lopez and Morrison look like a narrow change; the Gun-Free School Zones Act was easily amended, and lower courts accepted the fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="112" t="inlineStr">
+        <is>
+          <t>NFIB v. Sebelius: how to read the opinion</t>
+        </is>
+      </c>
+      <c r="B3" s="111" t="inlineStr">
+        <is>
+          <t>• Multiple holdings; not a typical opinion, so you can't just count votes.
+• Five Justices (Roberts plus the four dissenters) agreed the Commerce Clause doesn't support the individual mandate, but the dissenters didn't join Roberts's opinion, so that point may be dicta.
+• Five Justices upheld the mandate under the taxing power.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="112" t="inlineStr">
+        <is>
+          <t>NFIB: the activity/inactivity line</t>
+        </is>
+      </c>
+      <c r="B4" s="111" t="inlineStr">
+        <is>
+          <t>• Roberts: Congress can regulate people already in a market, but can't force people into commerce they're not engaged in.
+• The target: young, healthy people who weren't buying insurance.
+• Ginsburg: everyone participates in health care eventually, so this market is different.
+• Roberts: everyone will buy food, clothing and shelter too, but that doesn't let Congress order purchases; the Commerce Clause isn't a license to regulate a person 'from cradle to grave.' Police power over individuals stays with the States.
+• The federal government has only enumerated powers; if Congress can make you buy this, maybe there's no line (though cases like Hodel suggest the limits were reached long ago).
+• The line is hard to draw, but the Court is trying to draw a practical one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="112" t="inlineStr">
+        <is>
+          <t>NFIB: the mandate as a tax (Drexel Furniture)</t>
+        </is>
+      </c>
+      <c r="B5" s="111" t="inlineStr">
+        <is>
+          <t>• Labels don't matter; the taxing power is very broad but not unlimited.
+• Drexel Furniture (child labor 'tax') was really a penalty: (1) a crushing burden (10% of net income) for any violation, (2) only on those who knowingly hired children (scienter), (3) enforced partly by the Labor Department.
+• Background: before 1937 (Hammer), Congress couldn't regulate child labor because manufacturing came before commerce, so it tried the taxing power to punish what it couldn't reach directly.
+• The shared responsibility payment is different: usually less than insurance (can never be more), no scienter requirement, and collected only by the IRS through normal tax means (no criminal prosecution).
+• So it's a tax, not a punishment; five votes uphold the mandate this way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="112" t="inlineStr">
+        <is>
+          <t>NFIB: Medicaid expansion and Dole</t>
+        </is>
+      </c>
+      <c r="B6" s="111" t="inlineStr">
+        <is>
+          <t>• States had to change their Medicaid programs or lose ALL their existing Medicaid funds.
+• South Dakota v. Dole: raise the drinking age to 21 or lose 5% of highway funds; upheld. General welfare, clear terms, no other constitutional bar; the dissent said the link to highway funds was too attenuated, the majority found a plausible connection.
+• Incentives can go too far and become coercive: Roberts called the Medicaid threat 'a gun to the head.'
+• In Dole States could say no; as a practical matter, they couldn't refuse Medicaid funds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="112" t="inlineStr">
+        <is>
+          <t>The spectrum of views on federal power</t>
+        </is>
+      </c>
+      <c r="B7" s="111" t="inlineStr">
+        <is>
+          <t>• Broadest: Ginsburg (dissented in Lopez and Morrison, in the Raich majority).
+• Narrowest: Thomas (Lopez concurrence; narrowest view of the Commerce Clause of any Justice).
+• Underlying question: are there any real limits?</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="112" t="inlineStr">
+        <is>
+          <t>U.S. v. Phomma: the jurisdictional hook</t>
+        </is>
+      </c>
+      <c r="B8" s="111" t="inlineStr">
+        <is>
+          <t>• Not binding precedent. Civil disorder statute (18 U.S.C. §231): obstructing law enforcement or firefighters during a civil disorder; seems very broad (even 'delays').
+• Focus on Lopez category 3 (substantially affects commerce): can Congress criminalize obstructing or delaying a delivery vehicle? Yes, because of the jurisdictional hook (from Lopez), citing Dorsey.
+• Dorsey (9th Cir.): once Clinton's amendment added a commerce hook to the Gun-Free School Zones Act, prosecutions continued.
+• The hook must be substantive, not added just to ward off Commerce Clause challenges.
+• After Dorsey, Lopez looks like 'a big nothing' that is easy to get around.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="112" t="inlineStr">
+        <is>
+          <t>U.S. v. Protho (7th Cir. 2022): instrumentalities</t>
+        </is>
+      </c>
+      <c r="B9" s="111" t="inlineStr">
+        <is>
+          <t>• Protho argued the prosecution offered no evidence linking his act to interstate commerce.
+• Lopez category 1/2: protecting instrumentalities of interstate commerce. Federal Kidnapping Act; a car was used in the crime.
+• The court treated automobiles as a class as instrumentalities (many circuits agree; Morgan, 10th Cir.: cell phones, internet and GPS too).
+• Worry: if these courts are right, Congress could reach almost any crime, even without a gun that once crossed state lines. 'Motor vehicles' is broader than 'automobiles.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="112" t="inlineStr">
+        <is>
+          <t>U.S. v. Chavarria (10th Cir. 2025): the other side</t>
+        </is>
+      </c>
+      <c r="B10" s="111" t="inlineStr">
+        <is>
+          <t>• Kidnapping and murder in New Mexico; the problem was the indictment.
+• Some circuits treat motor vehicles as a class as instrumentalities (cars, even scooters); others don't. The Supreme Court has never defined 'instrumentalities of commerce.'
+• Tenth Circuit: instrumentalities are the means of interstate commerce (ships, railroads); motor vehicles are NOT always presumed to be instrumentalities.
+• Footnote: Congress might reach kidnapping under category 3 (aggregation, Wickard), but the statute didn't rely on that and the government didn't argue it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="112" t="inlineStr">
+        <is>
+          <t>Takeaway on Commerce Clause limits; Bonner</t>
+        </is>
+      </c>
+      <c r="B11" s="111" t="inlineStr">
+        <is>
+          <t>• Once the government jumps through jurisdictional hoops, there's little it can't regulate; a phone, the internet or a car can serve as the hook.
+• The Commerce Clause remains extraordinarily broad.
+• Bonner (Willett concurrence) worries lower courts have read the commerce power too broadly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="112" t="inlineStr">
+        <is>
+          <t>Brutus vs. Madison (Federalist 44) on Necessary and Proper</t>
+        </is>
+      </c>
+      <c r="B12" s="111" t="inlineStr">
+        <is>
+          <t>• Anti-Federalist fear (Brutus): Article I, §8 powers, especially Necessary and Proper, would be read so broadly they'd swallow the States.
+• Madison (Fed. 44): no part is more 'invulnerable.' The Convention's other options: (1) copy the Articles' 'expressly delegated' limit, (2) list every implied power, (3) list the excluded powers, or (4) say nothing and leave it to inference.
+• Copying the Articles meant a weak central government, which wasn't popular. No perfect solution to how explicit the grants must be.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="112" t="inlineStr">
+        <is>
+          <t>Tenth Amendment: 'expressly' left out</t>
+        </is>
+      </c>
+      <c r="B13" s="111" t="inlineStr">
+        <is>
+          <t>• Articles of Confederation, Art. II: States keep every power not 'expressly delegated.' The Tenth Amendment drops 'expressly.'
+• Not an oversight: proposals to add 'expressly' were voted down twice.
+• Madison: impossible to confine a government to express powers; implied powers are necessary unless the Constitution listed every detail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="112" t="inlineStr">
+        <is>
+          <t>The bank debate (1791): Madison vs. Ames</t>
+        </is>
+      </c>
+      <c r="B14" s="111" t="inlineStr">
+        <is>
+          <t>• Madison (then in Congress) argued Congress lacked power to charter a bank: no clause (taxing/general welfare, borrowing, or Necessary and Proper) supports it. Article I, §8 lists subsidiary powers (e.g., raising armies alongside declaring war), which counsels against stretching implied powers. A bank might just be 'convenient.'
+• Fisher Ames (Federalist, Massachusetts): being at the Convention doesn't make Madison right; it's too late to deny powers 'plainly implied.' Congress may do what's necessary to the Constitution's ends unless it violates rights, express reservations, or States' powers (similar to Marshall later).
+• Privately, Ames said the constitutional argument was 'a dull piece of business'; the real fight was where the capital would be. Philadelphia (with the bank) vs. moving the capital south, favored by the Virginians (Washington, Jefferson, Madison).
+• 1816: President Madison signed the Second Bank bill to deal with economic and currency problems after the first bank expired.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="112" t="inlineStr">
+        <is>
+          <t>McCulloch v. Maryland (1819): who created the Union</t>
+        </is>
+      </c>
+      <c r="B15" s="111" t="inlineStr">
+        <is>
+          <t>• Second Bank; Maryland taxed it. Two questions: can Congress charter a bank, and can Maryland tax it?
+• Historical practice matters to Marshall: this was the second bank; Washington, persuaded by Hamilton, signed the first.
+• Maryland argued the States created the federal government, so federal power should be read narrowly and in subordination to the States.
+• Marshall rejected that: the people created the federal government, so its powers needn't be construed strictly. It's a government of enumerated powers, but how far those powers reach will always be debated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="112" t="inlineStr">
+        <is>
+          <t>McCulloch: 'necessary' and the test</t>
+        </is>
+      </c>
+      <c r="B16" s="111" t="inlineStr">
+        <is>
+          <t>• The power to charter a bank comes from Article I, §8 through the Necessary and Proper Clause.
+• 'Necessary' doesn't mean absolutely necessary; it means convenient, useful (para. 27). Textual point: if the ratifiers wanted a strict limit, they could have worded it differently.
+• The test (para. 38): 'Let the end be legitimate, let it be within the scope of the constitution, and all means which are appropriate, which are plainly adapted to that end, which are not prohibited, but consist with the letter and spirit of the constitution, are constitutional.' Much like Ames.
+• The Tenth Amendment's missing 'expressly' means it doesn't block this. The bank is constitutional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="112" t="inlineStr">
+        <is>
+          <t>McCulloch: Maryland can't tax the bank; big picture</t>
+        </is>
+      </c>
+      <c r="B17" s="111" t="inlineStr">
+        <is>
+          <t>• 'The power to tax involves the power to destroy'; one government can't control the constitutional measures of the supreme one. Relying on 'confidence' that a State won't abuse the tax isn't enough.
+• Big takeaway: read federal power broadly. Hamiltonian view; broad Necessary and Proper Clause. Congress may do what's convenient to carry out its powers as long as it doesn't violate the Constitution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="112" t="inlineStr">
+        <is>
+          <t>Dormant Commerce Clause: origins and two tiers</t>
+        </is>
+      </c>
+      <c r="B18" s="111" t="inlineStr">
+        <is>
+          <t>• Hamilton (Fed. 11) wanted free trade within the U.S. and to avoid trade wars between States; Madison said giving Congress commerce power was uncontroversial.
+• Dormant Commerce Clause: even when Congress is silent, States can violate the Commerce Clause. Unusual for an Article I, §8 power.
+• Brown-Forman (1986): two tiers. (1) Laws that directly regulate or discriminate against interstate commerce, or favor in-state interests, are generally struck down. (2) Evenhanded laws with indirect effects get Pike balancing. No clear line between the two; the key is the overall effect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="112" t="inlineStr">
+        <is>
+          <t>Dean Milk and Pike</t>
+        </is>
+      </c>
+      <c r="B19" s="111" t="inlineStr">
+        <is>
+          <t>• Dean Milk (Madison, WI): milk had to be pasteurized within 5 miles and come from within 25 miles; an Illinois processor sued. Congress was silent, so it's a dormant Commerce Clause case. (If Congress authorizes discrimination, States and cities may do it.)
+• Calling it a health measure doesn't save it; it doesn't matter that other Wisconsin milk was also excluded. It plainly discriminates, which isn't allowed if reasonable nondiscriminatory alternatives exist.
+• Pike v. Bruce Church (1970): Arizona required cantaloupes to be packed in Arizona (to stamp 'Arizona' on them) when the grower already had a California packing plant. Evenhanded laws with incidental effects are upheld unless the burden is clearly excessive compared with local benefits (a cost-benefit test).
+• Outright discrimination: strict test. Evenhanded: weigh costs and benefits.
+• National Pork Producers v. Ross (2023): read with the handout on the course site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="112" t="inlineStr">
+        <is>
+          <t>Two exceptions: Congress approves; market participant (Reeves)</t>
+        </is>
+      </c>
+      <c r="B20" s="111" t="inlineStr">
+        <is>
+          <t>• Exception 1: discrimination is allowed if Congress says so.
+• Exception 2 (Reeves v. Stake): South Dakota's state cement plant supplied in-state customers first during a shortage; allowed because the State acted as a market participant, not a regulator. In-state tuition is analogous.
+• Hoarding a limited natural resource could come out differently.</t>
         </is>
       </c>
     </row>

</xml_diff>